<commit_message>
Ahora exporta nombres y Cuadrillas, tambien calcula MES y AÑO desde plantilla Excel
</commit_message>
<xml_diff>
--- a/models/he_2026_plantilla.xlsx
+++ b/models/he_2026_plantilla.xlsx
@@ -21,8 +21,8 @@
     <definedName function="false" hidden="false" name="_Key1" vbProcedure="false">NA()</definedName>
     <definedName function="false" hidden="false" name="_Order1" vbProcedure="false">255</definedName>
     <definedName function="false" hidden="false" name="_Sort" vbProcedure="false">NA()</definedName>
-    <definedName function="false" hidden="false" name="_xlfn_IFERROR" vbProcedure="false">#ref!</definedName>
-    <definedName function="false" hidden="false" name="_xlfn__FV" vbProcedure="false">#ref!</definedName>
+    <definedName function="false" hidden="false" name="_xlfn_IFERROR" vbProcedure="false">#REF!</definedName>
+    <definedName function="false" hidden="false" name="_xlfn__FV" vbProcedure="false">#REF!</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="Imprimir_títulos_IM" vbProcedure="false">NA()</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="Imprimir_área_IM" vbProcedure="false">NA()</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_Regression_Int" vbProcedure="false">1</definedName>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="88">
   <si>
     <t xml:space="preserve">Aplica</t>
   </si>
@@ -247,9 +247,6 @@
   </si>
   <si>
     <t xml:space="preserve">Parte:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ABRIL 2026</t>
   </si>
   <si>
     <t xml:space="preserve">                      Trabajador                                                                    Jefe Zonal                                                                Ingeniero 1                </t>
@@ -1693,12 +1690,13 @@
       <c r="E3" s="33"/>
       <c r="F3" s="33"/>
       <c r="G3" s="33"/>
-      <c r="H3" s="22" t="s">
-        <v>70</v>
+      <c r="H3" s="22" t="str">
+        <f aca="false">UPPER(TEXT(B6, "mmmm yyyy"))</f>
+        <v>ABRIL 2026</v>
       </c>
       <c r="I3" s="34"/>
       <c r="J3" s="35" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K3" s="18"/>
       <c r="L3" s="18"/>
@@ -1734,34 +1732,34 @@
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="40" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="41" t="s">
         <v>72</v>
       </c>
-      <c r="B5" s="41" t="s">
+      <c r="C5" s="40" t="s">
         <v>73</v>
       </c>
-      <c r="C5" s="40" t="s">
+      <c r="D5" s="40" t="s">
         <v>74</v>
       </c>
-      <c r="D5" s="40" t="s">
+      <c r="E5" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="E5" s="40" t="s">
+      <c r="F5" s="41" t="s">
         <v>76</v>
       </c>
-      <c r="F5" s="41" t="s">
+      <c r="G5" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="G5" s="40" t="s">
+      <c r="H5" s="40" t="s">
         <v>78</v>
       </c>
-      <c r="H5" s="40" t="s">
+      <c r="I5" s="40" t="s">
         <v>79</v>
       </c>
-      <c r="I5" s="40" t="s">
+      <c r="J5" s="40" t="s">
         <v>80</v>
-      </c>
-      <c r="J5" s="40" t="s">
-        <v>81</v>
       </c>
       <c r="K5" s="42"/>
       <c r="L5" s="42"/>
@@ -2056,7 +2054,7 @@
         <v>0.0618055555555556</v>
       </c>
       <c r="J7" s="52" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="R7" s="36"/>
       <c r="S7" s="31"/>
@@ -2089,7 +2087,7 @@
         <v>0.268055555555556</v>
       </c>
       <c r="J8" s="52" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="R8" s="36"/>
       <c r="S8" s="31"/>
@@ -2118,7 +2116,7 @@
         <v>0.0888888888888889</v>
       </c>
       <c r="J9" s="52" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="R9" s="36"/>
       <c r="S9" s="31"/>
@@ -2147,7 +2145,7 @@
         <v>0.0840277777777778</v>
       </c>
       <c r="J10" s="52" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="R10" s="36"/>
       <c r="S10" s="31"/>
@@ -2176,7 +2174,7 @@
         <v>0.0868055555555556</v>
       </c>
       <c r="J11" s="52" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="R11" s="36"/>
       <c r="S11" s="31"/>
@@ -2205,7 +2203,7 @@
         <v>0.0972222222222222</v>
       </c>
       <c r="J12" s="52" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="R12" s="36"/>
       <c r="S12" s="31"/>
@@ -2280,7 +2278,7 @@
         <v>0.0902777777777778</v>
       </c>
       <c r="J15" s="52" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="R15" s="36"/>
       <c r="S15" s="31"/>
@@ -5187,7 +5185,7 @@
   <pageMargins left="0.669444444444445" right="0.669444444444445" top="0.865972222222222" bottom="0.227083333333333" header="0.196527777777778" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="61" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Aptos,Normal"&amp;16GERENCIA DE OPERACIÓN Y MANTENIMIENTO
+    <oddHeader>&amp;C&amp;"Aptos,Regular"&amp;16GERENCIA DE OPERACIÓN Y MANTENIMIENTO
 &amp;12SUPERINTENDENCIA DE OPERACIÓN Y MANTENIMIENTO ZONA 1
 Reporte Horas Extraordinarias </oddHeader>
     <oddFooter/>

</xml_diff>

<commit_message>
BUG no procesa bien las ot del 30 de abril, manteiene el TimeZone y no reconoce como Fecha - MIGRAR a DuckDB
</commit_message>
<xml_diff>
--- a/models/he_2026_plantilla.xlsx
+++ b/models/he_2026_plantilla.xlsx
@@ -20,8 +20,8 @@
     <definedName function="false" hidden="false" name="_Key1" vbProcedure="false">NA()</definedName>
     <definedName function="false" hidden="false" name="_Order1" vbProcedure="false">255</definedName>
     <definedName function="false" hidden="false" name="_Sort" vbProcedure="false">NA()</definedName>
-    <definedName function="false" hidden="false" name="_xlfn_IFERROR" vbProcedure="false">#REF!</definedName>
-    <definedName function="false" hidden="false" name="_xlfn__FV" vbProcedure="false">#REF!</definedName>
+    <definedName function="false" hidden="false" name="_xlfn_IFERROR" vbProcedure="false">#ref!</definedName>
+    <definedName function="false" hidden="false" name="_xlfn__FV" vbProcedure="false">#ref!</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="Imprimir_títulos_IM" vbProcedure="false">NA()</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="Imprimir_área_IM" vbProcedure="false">NA()</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_Regression_Int" vbProcedure="false">1</definedName>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <r>
       <rPr>
@@ -136,16 +136,20 @@
   <si>
     <t xml:space="preserve">OT # 174486.Tutus, Est 91980 cambio de tirafusible 12A-T</t>
   </si>
+  <si>
+    <t xml:space="preserve">Calle Atahualpa - Velazco Ibarra, red de baja tensión arrancada por corto circuito. se recupera conductor en buen estado, se usa 3 varillas #2 y 1/0 de empalme en 5005 y acsr.....</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
-    <numFmt numFmtId="166" formatCode="h:mm;@"/>
-    <numFmt numFmtId="167" formatCode="[$-C0A]d/mmm\ yyyy;@"/>
+    <numFmt numFmtId="166" formatCode="h:mm"/>
+    <numFmt numFmtId="167" formatCode="h:mm;@"/>
+    <numFmt numFmtId="168" formatCode="[$-C0A]d/mmm\ yyyy;@"/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -573,7 +577,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -633,19 +637,19 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -653,15 +657,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -669,23 +673,23 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -796,9 +800,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>111240</xdr:colOff>
+      <xdr:colOff>110520</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>1056240</xdr:rowOff>
+      <xdr:rowOff>1055520</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -812,7 +816,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2040480" cy="1056240"/>
+          <a:ext cx="2039760" cy="1055520"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -834,9 +838,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>7872120</xdr:colOff>
+      <xdr:colOff>7871400</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>401760</xdr:rowOff>
+      <xdr:rowOff>401040</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -850,7 +854,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10395360" y="21960"/>
-          <a:ext cx="4151880" cy="379800"/>
+          <a:ext cx="4151160" cy="379080"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1040,8 +1044,8 @@
         <v>5</v>
       </c>
       <c r="I3" s="12" t="n">
-        <f aca="false">SUM(I6:I36)*24</f>
-        <v>18.65</v>
+        <f aca="false">SUM(I6:I36)</f>
+        <v>0.777083333333334</v>
       </c>
       <c r="J3" s="13" t="s">
         <v>6</v>
@@ -1544,7 +1548,7 @@
       </c>
       <c r="J25" s="35"/>
     </row>
-    <row r="26" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="27" t="str">
         <f aca="false">IF(B26&gt;0,PROPER(TEXT(B26,"dddd")),"")</f>
         <v>Martes</v>
@@ -1562,7 +1566,9 @@
         <f aca="false">SUM(C26:H26)</f>
         <v>0</v>
       </c>
-      <c r="J26" s="35"/>
+      <c r="J26" s="35" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="27" t="str">

</xml_diff>

<commit_message>
Funciona, hay q probar cargando más Ordenes de Trabajo
</commit_message>
<xml_diff>
--- a/models/he_2026_plantilla.xlsx
+++ b/models/he_2026_plantilla.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <r>
       <rPr>
@@ -135,9 +135,6 @@
   </si>
   <si>
     <t xml:space="preserve">OT # 174486.Tutus, Est 91980 cambio de tirafusible 12A-T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calle Atahualpa - Velazco Ibarra, red de baja tensión arrancada por corto circuito. se recupera conductor en buen estado, se usa 3 varillas #2 y 1/0 de empalme en 5005 y acsr.....</t>
   </si>
 </sst>
 </file>
@@ -447,16 +444,16 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
-      <right style="thin">
-        <color rgb="FF3465A4"/>
-      </right>
+      <right/>
       <top/>
       <bottom style="thin"/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
-      <right/>
+      <right style="thin">
+        <color rgb="FF3465A4"/>
+      </right>
       <top/>
       <bottom style="thin"/>
       <diagonal/>
@@ -528,7 +525,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -681,15 +678,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="167" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="15" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -800,9 +793,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>110520</xdr:colOff>
+      <xdr:colOff>109800</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>1055520</xdr:rowOff>
+      <xdr:rowOff>1054800</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -816,7 +809,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2039760" cy="1055520"/>
+          <a:ext cx="2039040" cy="1054800"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -838,9 +831,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>7871400</xdr:colOff>
+      <xdr:colOff>7870680</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>401040</xdr:rowOff>
+      <xdr:rowOff>400320</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -854,7 +847,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="10395360" y="21960"/>
-          <a:ext cx="4151160" cy="379080"/>
+          <a:ext cx="4150440" cy="378360"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1024,7 +1017,7 @@
       </c>
       <c r="I2" s="8" t="n">
         <f aca="false">SUM(K6:K36)</f>
-        <v>0</v>
+        <v>33.0166666666667</v>
       </c>
       <c r="J2" s="9" t="s">
         <v>3</v>
@@ -1067,7 +1060,7 @@
       <c r="G4" s="16"/>
       <c r="H4" s="17" t="str">
         <f aca="false">UPPER(TEXT(B6, "mmmm aaaa"))</f>
-        <v>ABRIL 2026</v>
+        <v>MAYO 2026</v>
       </c>
       <c r="I4" s="18"/>
       <c r="J4" s="19" t="s">
@@ -1117,10 +1110,10 @@
     <row r="6" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="27" t="str">
         <f aca="false">IF(B6&gt;0,PROPER(TEXT(B6,"dddd")),"")</f>
-        <v>Miércoles</v>
+        <v>Viernes</v>
       </c>
       <c r="B6" s="28" t="n">
-        <v>46113</v>
+        <v>46143</v>
       </c>
       <c r="C6" s="29"/>
       <c r="D6" s="30"/>
@@ -1132,14 +1125,18 @@
         <v>0</v>
       </c>
       <c r="J6" s="31"/>
+      <c r="K6" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*2*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="27" t="str">
         <f aca="false">IF(B7&gt;0,PROPER(TEXT(B7,"dddd")),"")</f>
-        <v>Jueves</v>
+        <v>Sábado</v>
       </c>
       <c r="B7" s="32" t="n">
-        <v>46114</v>
+        <v>46144</v>
       </c>
       <c r="C7" s="33" t="n">
         <v>0.803472222222222</v>
@@ -1157,14 +1154,18 @@
       <c r="J7" s="35" t="s">
         <v>19</v>
       </c>
+      <c r="K7" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*2*24)</f>
+        <v>2.96666666666669</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="str">
         <f aca="false">IF(B8&gt;0,PROPER(TEXT(B8,"dddd")),"")</f>
-        <v>Viernes</v>
+        <v>Domingo</v>
       </c>
       <c r="B8" s="32" t="n">
-        <v>46115</v>
+        <v>46145</v>
       </c>
       <c r="C8" s="33" t="n">
         <v>0.370138888888889</v>
@@ -1186,14 +1187,18 @@
       <c r="J8" s="35" t="s">
         <v>20</v>
       </c>
+      <c r="K8" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*2*24)</f>
+        <v>12.8666666666666</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="27" t="str">
         <f aca="false">IF(B9&gt;0,PROPER(TEXT(B9,"dddd")),"")</f>
-        <v>Sábado</v>
-      </c>
-      <c r="B9" s="32" t="n">
-        <v>46116</v>
+        <v>Lunes</v>
+      </c>
+      <c r="B9" s="28" t="n">
+        <v>46146</v>
       </c>
       <c r="C9" s="33" t="n">
         <v>0.677777777777778</v>
@@ -1211,14 +1216,18 @@
       <c r="J9" s="35" t="s">
         <v>21</v>
       </c>
+      <c r="K9" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>3.2</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="27" t="str">
         <f aca="false">IF(B10&gt;0,PROPER(TEXT(B10,"dddd")),"")</f>
-        <v>Domingo</v>
+        <v>Martes</v>
       </c>
       <c r="B10" s="32" t="n">
-        <v>46117</v>
+        <v>46147</v>
       </c>
       <c r="C10" s="33" t="n">
         <v>0.366666666666667</v>
@@ -1236,14 +1245,18 @@
       <c r="J10" s="35" t="s">
         <v>22</v>
       </c>
+      <c r="K10" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>3.02499999999997</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="27" t="str">
         <f aca="false">IF(B11&gt;0,PROPER(TEXT(B11,"dddd")),"")</f>
-        <v>Lunes</v>
+        <v>Miércoles</v>
       </c>
       <c r="B11" s="32" t="n">
-        <v>46118</v>
+        <v>46148</v>
       </c>
       <c r="C11" s="33" t="n">
         <v>0.798611111111111</v>
@@ -1261,14 +1274,18 @@
       <c r="J11" s="35" t="s">
         <v>23</v>
       </c>
+      <c r="K11" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>3.12500000000001</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="27" t="str">
         <f aca="false">IF(B12&gt;0,PROPER(TEXT(B12,"dddd")),"")</f>
-        <v>Martes</v>
-      </c>
-      <c r="B12" s="32" t="n">
-        <v>46119</v>
+        <v>Jueves</v>
+      </c>
+      <c r="B12" s="28" t="n">
+        <v>46149</v>
       </c>
       <c r="C12" s="33" t="n">
         <v>0.75</v>
@@ -1286,14 +1303,18 @@
       <c r="J12" s="35" t="s">
         <v>24</v>
       </c>
+      <c r="K12" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>3.49999999999999</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="27" t="str">
         <f aca="false">IF(B13&gt;0,PROPER(TEXT(B13,"dddd")),"")</f>
-        <v>Miércoles</v>
+        <v>Viernes</v>
       </c>
       <c r="B13" s="32" t="n">
-        <v>46120</v>
+        <v>46150</v>
       </c>
       <c r="C13" s="33"/>
       <c r="D13" s="34"/>
@@ -1305,14 +1326,18 @@
         <v>0</v>
       </c>
       <c r="J13" s="35"/>
+      <c r="K13" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="27" t="str">
         <f aca="false">IF(B14&gt;0,PROPER(TEXT(B14,"dddd")),"")</f>
-        <v>Jueves</v>
+        <v>Sábado</v>
       </c>
       <c r="B14" s="32" t="n">
-        <v>46121</v>
+        <v>46151</v>
       </c>
       <c r="C14" s="33"/>
       <c r="D14" s="34"/>
@@ -1324,14 +1349,18 @@
         <v>0</v>
       </c>
       <c r="J14" s="35"/>
+      <c r="K14" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*2*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="27" t="str">
         <f aca="false">IF(B15&gt;0,PROPER(TEXT(B15,"dddd")),"")</f>
-        <v>Viernes</v>
-      </c>
-      <c r="B15" s="32" t="n">
-        <v>46122</v>
+        <v>Domingo</v>
+      </c>
+      <c r="B15" s="28" t="n">
+        <v>46152</v>
       </c>
       <c r="C15" s="33" t="n">
         <v>0.727083333333333</v>
@@ -1349,14 +1378,18 @@
       <c r="J15" s="35" t="s">
         <v>25</v>
       </c>
+      <c r="K15" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*2*24)</f>
+        <v>4.33333333333335</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27" t="str">
         <f aca="false">IF(B16&gt;0,PROPER(TEXT(B16,"dddd")),"")</f>
-        <v>Sábado</v>
+        <v>Lunes</v>
       </c>
       <c r="B16" s="32" t="n">
-        <v>46123</v>
+        <v>46153</v>
       </c>
       <c r="C16" s="33"/>
       <c r="D16" s="34"/>
@@ -1368,14 +1401,18 @@
         <v>0</v>
       </c>
       <c r="J16" s="35"/>
+      <c r="K16" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="27" t="str">
         <f aca="false">IF(B17&gt;0,PROPER(TEXT(B17,"dddd")),"")</f>
-        <v>Domingo</v>
+        <v>Martes</v>
       </c>
       <c r="B17" s="32" t="n">
-        <v>46124</v>
+        <v>46154</v>
       </c>
       <c r="C17" s="33"/>
       <c r="D17" s="34"/>
@@ -1387,14 +1424,18 @@
         <v>0</v>
       </c>
       <c r="J17" s="35"/>
+      <c r="K17" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="27" t="str">
         <f aca="false">IF(B18&gt;0,PROPER(TEXT(B18,"dddd")),"")</f>
-        <v>Lunes</v>
-      </c>
-      <c r="B18" s="32" t="n">
-        <v>46125</v>
+        <v>Miércoles</v>
+      </c>
+      <c r="B18" s="28" t="n">
+        <v>46155</v>
       </c>
       <c r="C18" s="33"/>
       <c r="D18" s="34"/>
@@ -1407,14 +1448,18 @@
         <v>0</v>
       </c>
       <c r="J18" s="35"/>
+      <c r="K18" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="27" t="str">
         <f aca="false">IF(B19&gt;0,PROPER(TEXT(B19,"dddd")),"")</f>
-        <v>Martes</v>
+        <v>Jueves</v>
       </c>
       <c r="B19" s="32" t="n">
-        <v>46126</v>
+        <v>46156</v>
       </c>
       <c r="C19" s="33"/>
       <c r="D19" s="34"/>
@@ -1427,14 +1472,18 @@
         <v>0</v>
       </c>
       <c r="J19" s="35"/>
+      <c r="K19" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="27" t="str">
         <f aca="false">IF(B20&gt;0,PROPER(TEXT(B20,"dddd")),"")</f>
-        <v>Miércoles</v>
+        <v>Viernes</v>
       </c>
       <c r="B20" s="32" t="n">
-        <v>46127</v>
+        <v>46157</v>
       </c>
       <c r="C20" s="33"/>
       <c r="D20" s="34"/>
@@ -1447,14 +1496,18 @@
         <v>0</v>
       </c>
       <c r="J20" s="35"/>
+      <c r="K20" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="27" t="str">
         <f aca="false">IF(B21&gt;0,PROPER(TEXT(B21,"dddd")),"")</f>
-        <v>Jueves</v>
-      </c>
-      <c r="B21" s="32" t="n">
-        <v>46128</v>
+        <v>Sábado</v>
+      </c>
+      <c r="B21" s="28" t="n">
+        <v>46158</v>
       </c>
       <c r="C21" s="33"/>
       <c r="D21" s="34"/>
@@ -1467,14 +1520,18 @@
         <v>0</v>
       </c>
       <c r="J21" s="35"/>
+      <c r="K21" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*2*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="27" t="str">
         <f aca="false">IF(B22&gt;0,PROPER(TEXT(B22,"dddd")),"")</f>
-        <v>Viernes</v>
+        <v>Domingo</v>
       </c>
       <c r="B22" s="32" t="n">
-        <v>46129</v>
+        <v>46159</v>
       </c>
       <c r="C22" s="33"/>
       <c r="D22" s="34"/>
@@ -1487,14 +1544,18 @@
         <v>0</v>
       </c>
       <c r="J22" s="35"/>
+      <c r="K22" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*2*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="27" t="str">
         <f aca="false">IF(B23&gt;0,PROPER(TEXT(B23,"dddd")),"")</f>
-        <v>Sábado</v>
+        <v>Lunes</v>
       </c>
       <c r="B23" s="32" t="n">
-        <v>46130</v>
+        <v>46160</v>
       </c>
       <c r="C23" s="33"/>
       <c r="D23" s="34"/>
@@ -1507,14 +1568,18 @@
         <v>0</v>
       </c>
       <c r="J23" s="35"/>
+      <c r="K23" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="27" t="str">
         <f aca="false">IF(B24&gt;0,PROPER(TEXT(B24,"dddd")),"")</f>
-        <v>Domingo</v>
-      </c>
-      <c r="B24" s="32" t="n">
-        <v>46131</v>
+        <v>Martes</v>
+      </c>
+      <c r="B24" s="28" t="n">
+        <v>46161</v>
       </c>
       <c r="C24" s="33"/>
       <c r="D24" s="34"/>
@@ -1527,14 +1592,18 @@
         <v>0</v>
       </c>
       <c r="J24" s="35"/>
+      <c r="K24" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="27" t="str">
         <f aca="false">IF(B25&gt;0,PROPER(TEXT(B25,"dddd")),"")</f>
-        <v>Lunes</v>
+        <v>Miércoles</v>
       </c>
       <c r="B25" s="32" t="n">
-        <v>46132</v>
+        <v>46162</v>
       </c>
       <c r="C25" s="33"/>
       <c r="D25" s="34"/>
@@ -1547,14 +1616,18 @@
         <v>0</v>
       </c>
       <c r="J25" s="35"/>
-    </row>
-    <row r="26" customFormat="false" ht="20.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="K25" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="27" t="str">
         <f aca="false">IF(B26&gt;0,PROPER(TEXT(B26,"dddd")),"")</f>
-        <v>Martes</v>
+        <v>Jueves</v>
       </c>
       <c r="B26" s="32" t="n">
-        <v>46133</v>
+        <v>46163</v>
       </c>
       <c r="C26" s="33"/>
       <c r="D26" s="34"/>
@@ -1566,17 +1639,19 @@
         <f aca="false">SUM(C26:H26)</f>
         <v>0</v>
       </c>
-      <c r="J26" s="35" t="s">
-        <v>26</v>
+      <c r="J26" s="35"/>
+      <c r="K26" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="27" t="str">
         <f aca="false">IF(B27&gt;0,PROPER(TEXT(B27,"dddd")),"")</f>
-        <v>Miércoles</v>
-      </c>
-      <c r="B27" s="32" t="n">
-        <v>46134</v>
+        <v>Viernes</v>
+      </c>
+      <c r="B27" s="28" t="n">
+        <v>46164</v>
       </c>
       <c r="C27" s="33"/>
       <c r="D27" s="34"/>
@@ -1589,14 +1664,18 @@
         <v>0</v>
       </c>
       <c r="J27" s="35"/>
+      <c r="K27" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="27" t="str">
         <f aca="false">IF(B28&gt;0,PROPER(TEXT(B28,"dddd")),"")</f>
-        <v>Jueves</v>
+        <v>Sábado</v>
       </c>
       <c r="B28" s="32" t="n">
-        <v>46135</v>
+        <v>46165</v>
       </c>
       <c r="C28" s="33"/>
       <c r="D28" s="34"/>
@@ -1609,14 +1688,18 @@
         <v>0</v>
       </c>
       <c r="J28" s="35"/>
+      <c r="K28" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*2*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="27" t="str">
         <f aca="false">IF(B29&gt;0,PROPER(TEXT(B29,"dddd")),"")</f>
-        <v>Viernes</v>
+        <v>Domingo</v>
       </c>
       <c r="B29" s="32" t="n">
-        <v>46136</v>
+        <v>46166</v>
       </c>
       <c r="C29" s="33"/>
       <c r="D29" s="34"/>
@@ -1629,14 +1712,18 @@
         <v>0</v>
       </c>
       <c r="J29" s="35"/>
+      <c r="K29" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*2*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="27" t="str">
         <f aca="false">IF(B30&gt;0,PROPER(TEXT(B30,"dddd")),"")</f>
-        <v>Sábado</v>
-      </c>
-      <c r="B30" s="32" t="n">
-        <v>46137</v>
+        <v>Lunes</v>
+      </c>
+      <c r="B30" s="28" t="n">
+        <v>46167</v>
       </c>
       <c r="C30" s="33"/>
       <c r="D30" s="34"/>
@@ -1649,14 +1736,18 @@
         <v>0</v>
       </c>
       <c r="J30" s="35"/>
+      <c r="K30" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="27" t="str">
         <f aca="false">IF(B31&gt;0,PROPER(TEXT(B31,"dddd")),"")</f>
-        <v>Domingo</v>
+        <v>Martes</v>
       </c>
       <c r="B31" s="32" t="n">
-        <v>46138</v>
+        <v>46168</v>
       </c>
       <c r="C31" s="33"/>
       <c r="D31" s="34"/>
@@ -1669,14 +1760,18 @@
         <v>0</v>
       </c>
       <c r="J31" s="35"/>
+      <c r="K31" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="27" t="str">
         <f aca="false">IF(B32&gt;0,PROPER(TEXT(B32,"dddd")),"")</f>
-        <v>Lunes</v>
+        <v>Miércoles</v>
       </c>
       <c r="B32" s="32" t="n">
-        <v>46139</v>
+        <v>46169</v>
       </c>
       <c r="C32" s="33"/>
       <c r="D32" s="34"/>
@@ -1689,14 +1784,18 @@
         <v>0</v>
       </c>
       <c r="J32" s="35"/>
+      <c r="K32" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="27" t="str">
         <f aca="false">IF(B33&gt;0,PROPER(TEXT(B33,"dddd")),"")</f>
-        <v>Martes</v>
-      </c>
-      <c r="B33" s="32" t="n">
-        <v>46140</v>
+        <v>Jueves</v>
+      </c>
+      <c r="B33" s="28" t="n">
+        <v>46170</v>
       </c>
       <c r="C33" s="33"/>
       <c r="D33" s="34"/>
@@ -1709,14 +1808,18 @@
         <v>0</v>
       </c>
       <c r="J33" s="35"/>
+      <c r="K33" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="27" t="str">
         <f aca="false">IF(B34&gt;0,PROPER(TEXT(B34,"dddd")),"")</f>
-        <v>Miércoles</v>
+        <v>Viernes</v>
       </c>
       <c r="B34" s="32" t="n">
-        <v>46141</v>
+        <v>46171</v>
       </c>
       <c r="C34" s="33"/>
       <c r="D34" s="34"/>
@@ -1729,14 +1832,18 @@
         <v>0</v>
       </c>
       <c r="J34" s="35"/>
+      <c r="K34" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*1.5*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="27" t="str">
         <f aca="false">IF(B35&gt;0,PROPER(TEXT(B35,"dddd")),"")</f>
-        <v>Jueves</v>
+        <v>Sábado</v>
       </c>
       <c r="B35" s="32" t="n">
-        <v>46142</v>
+        <v>46172</v>
       </c>
       <c r="C35" s="33"/>
       <c r="D35" s="34"/>
@@ -1749,36 +1856,46 @@
         <v>0</v>
       </c>
       <c r="J35" s="35"/>
+      <c r="K35" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*2*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="37" t="str">
         <f aca="false">IF(B36&gt;0,PROPER(TEXT(B36,"dddd")),"")</f>
-        <v/>
-      </c>
-      <c r="B36" s="38"/>
-      <c r="C36" s="39"/>
-      <c r="D36" s="40"/>
-      <c r="E36" s="39"/>
-      <c r="F36" s="40"/>
-      <c r="G36" s="39"/>
-      <c r="H36" s="40"/>
-      <c r="I36" s="39" t="n">
+        <v>Domingo</v>
+      </c>
+      <c r="B36" s="28" t="n">
+        <v>46173</v>
+      </c>
+      <c r="C36" s="38"/>
+      <c r="D36" s="39"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="39"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="39"/>
+      <c r="I36" s="38" t="n">
         <f aca="false">SUM(C36:H36)</f>
         <v>0</v>
       </c>
-      <c r="J36" s="41"/>
+      <c r="J36" s="40"/>
+      <c r="K36" s="1" t="n">
+        <f aca="true">SUMPRODUCT((INDIRECT({"D","F","H"}&amp;ROW())-INDIRECT({"C","E","G"}&amp;ROW()))*2*24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="42"/>
-      <c r="B37" s="43"/>
-      <c r="C37" s="43"/>
-      <c r="D37" s="43"/>
-      <c r="E37" s="43"/>
-      <c r="F37" s="43"/>
-      <c r="G37" s="43"/>
-      <c r="H37" s="43"/>
-      <c r="I37" s="44"/>
-      <c r="J37" s="43"/>
+      <c r="A37" s="41"/>
+      <c r="B37" s="42"/>
+      <c r="C37" s="42"/>
+      <c r="D37" s="42"/>
+      <c r="E37" s="42"/>
+      <c r="F37" s="42"/>
+      <c r="G37" s="42"/>
+      <c r="H37" s="42"/>
+      <c r="I37" s="43"/>
+      <c r="J37" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Se cambia el tipo de letra (ioskeva Extra Light Mono) para que el alto de la fila sea programatico segun el texto
</commit_message>
<xml_diff>
--- a/models/he_2026_plantilla.xlsx
+++ b/models/he_2026_plantilla.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/474e2f0e930ab59f/01 JEZO/temp_JEZO_borrar/0000 editar imagenes/reportes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="11_38B310D64F6F86F52E2977DC31515DFA2EEEB96F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AA25705-FBD8-4370-BB78-32CBD103C00B}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="11_38B310D64F6F86F52E2977DC31515DFA2EEEB96F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1581A79E-7F0A-437E-8D4D-0D01548B58B5}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25335" windowHeight="15465" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25350" windowHeight="15315" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HORAS_EXTRA" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <r>
       <rPr>
@@ -157,12 +157,6 @@
     <t>OT # 174080. FESTIVO. Naichap, restitución M# 194238 por 18-258039. Aguacate, restitución M# 194324 por 18-258040.</t>
   </si>
   <si>
-    <t>OT # 174083. Guayusal, Est 291765 cambio tirafusible 25A-T</t>
-  </si>
-  <si>
-    <t>OT # 174084. Chumpias, Est 028535 cambio tirafusible 25A-T</t>
-  </si>
-  <si>
     <t>OT # 174310. La Pradera, se arregla acometida M# 240908, se rehabilita trafo # 20916</t>
   </si>
   <si>
@@ -182,7 +176,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="h:mm;@"/>
     <numFmt numFmtId="165" formatCode="[$-C0A]d/mmm\ yyyy;@"/>
-    <numFmt numFmtId="168" formatCode="\(\ [h]:mm\ \)"/>
+    <numFmt numFmtId="166" formatCode="\(\ [h]:mm\ \)"/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -317,9 +311,8 @@
       <family val="3"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Nirmala UI Semilight"/>
-      <family val="2"/>
+      <sz val="9"/>
+      <name val="Iosevka Aile Extralight"/>
     </font>
   </fonts>
   <fills count="3">
@@ -336,7 +329,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -422,21 +415,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3465A4"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3465A4"/>
-      </top>
-      <bottom style="hair">
-        <color rgb="FF3465A4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color rgb="FF3465A4"/>
@@ -571,7 +549,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -635,22 +613,22 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -676,29 +654,26 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -886,6 +861,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -1011,18 +990,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="84.75" customHeight="1">
-      <c r="A1" s="40" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="40"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="40"/>
-      <c r="E1" s="40"/>
-      <c r="F1" s="40"/>
-      <c r="G1" s="40"/>
-      <c r="H1" s="40"/>
-      <c r="I1" s="40"/>
-      <c r="J1" s="40"/>
+      <c r="A1" s="42" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
     </row>
     <row r="2" spans="1:14" ht="21.75" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -1058,12 +1037,12 @@
       <c r="H3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="45">
+      <c r="I3" s="41">
         <f>SUM(I6:I36)</f>
         <v>1.3187500000000005</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="K3" s="11"/>
       <c r="L3" s="11"/>
@@ -1146,7 +1125,9 @@
       <c r="I6" s="21">
         <v>0</v>
       </c>
-      <c r="J6" s="41"/>
+      <c r="J6" s="43" t="s">
+        <v>18</v>
+      </c>
       <c r="K6" cm="1">
         <f t="array" aca="1" ref="K6" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*2*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*2*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*2*24)</f>
         <v>0</v>
@@ -1173,7 +1154,7 @@
       <c r="I7" s="24">
         <v>6.18055555555556E-2</v>
       </c>
-      <c r="J7" s="42" t="s">
+      <c r="J7" s="43" t="s">
         <v>18</v>
       </c>
       <c r="K7" cm="1">
@@ -1206,8 +1187,8 @@
       <c r="I8" s="24">
         <v>0.26805555555555599</v>
       </c>
-      <c r="J8" s="42" t="s">
-        <v>19</v>
+      <c r="J8" s="43" t="s">
+        <v>18</v>
       </c>
       <c r="K8" cm="1">
         <f t="array" aca="1" ref="K8" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*2*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*2*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*2*24)</f>
@@ -1235,8 +1216,8 @@
       <c r="I9" s="24">
         <v>8.8888888888888906E-2</v>
       </c>
-      <c r="J9" s="42" t="s">
-        <v>20</v>
+      <c r="J9" s="43" t="s">
+        <v>19</v>
       </c>
       <c r="K9" cm="1">
         <f t="array" aca="1" ref="K9" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
@@ -1264,8 +1245,8 @@
       <c r="I10" s="24">
         <v>8.4027777777777798E-2</v>
       </c>
-      <c r="J10" s="42" t="s">
-        <v>21</v>
+      <c r="J10" s="43" t="s">
+        <v>19</v>
       </c>
       <c r="K10" cm="1">
         <f t="array" aca="1" ref="K10" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
@@ -1293,8 +1274,8 @@
       <c r="I11" s="38">
         <v>8.6805555555555594E-2</v>
       </c>
-      <c r="J11" s="42" t="s">
-        <v>22</v>
+      <c r="J11" s="43" t="s">
+        <v>20</v>
       </c>
       <c r="K11" cm="1">
         <f t="array" aca="1" ref="K11" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
@@ -1322,8 +1303,8 @@
       <c r="I12" s="39">
         <v>9.7222222222222196E-2</v>
       </c>
-      <c r="J12" s="42" t="s">
-        <v>23</v>
+      <c r="J12" s="43" t="s">
+        <v>21</v>
       </c>
       <c r="K12" cm="1">
         <f t="array" aca="1" ref="K12" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
@@ -1347,7 +1328,7 @@
       <c r="I13" s="21">
         <v>0</v>
       </c>
-      <c r="J13" s="42"/>
+      <c r="J13" s="43"/>
       <c r="K13" cm="1">
         <f t="array" aca="1" ref="K13" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1370,7 +1351,7 @@
       <c r="I14" s="24">
         <v>0</v>
       </c>
-      <c r="J14" s="42"/>
+      <c r="J14" s="43"/>
       <c r="K14" cm="1">
         <f t="array" aca="1" ref="K14" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*2*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*2*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*2*24)</f>
         <v>0</v>
@@ -1397,8 +1378,8 @@
       <c r="I15" s="24">
         <v>9.0277777777777804E-2</v>
       </c>
-      <c r="J15" s="42" t="s">
-        <v>24</v>
+      <c r="J15" s="43" t="s">
+        <v>22</v>
       </c>
       <c r="K15" cm="1">
         <f t="array" aca="1" ref="K15" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*2*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*2*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*2*24)</f>
@@ -1422,7 +1403,7 @@
       <c r="I16" s="24">
         <v>0</v>
       </c>
-      <c r="J16" s="42"/>
+      <c r="J16" s="43"/>
       <c r="K16" cm="1">
         <f t="array" aca="1" ref="K16" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1450,7 +1431,7 @@
         <f>D17-C17</f>
         <v>0.54166666666666663</v>
       </c>
-      <c r="J17" s="42"/>
+      <c r="J17" s="43"/>
       <c r="K17" cm="1">
         <f t="array" aca="1" ref="K17" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>19.5</v>
@@ -1474,7 +1455,7 @@
         <f t="shared" ref="I18:I36" si="1">SUM(C18:H18)</f>
         <v>0</v>
       </c>
-      <c r="J18" s="42"/>
+      <c r="J18" s="43"/>
       <c r="K18" cm="1">
         <f t="array" aca="1" ref="K18" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1498,7 +1479,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J19" s="42"/>
+      <c r="J19" s="43"/>
       <c r="K19" cm="1">
         <f t="array" aca="1" ref="K19" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1522,7 +1503,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J20" s="42"/>
+      <c r="J20" s="43"/>
       <c r="K20" cm="1">
         <f t="array" aca="1" ref="K20" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1546,7 +1527,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J21" s="42"/>
+      <c r="J21" s="43"/>
       <c r="K21" cm="1">
         <f t="array" aca="1" ref="K21" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*2*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*2*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*2*24)</f>
         <v>0</v>
@@ -1570,7 +1551,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J22" s="42"/>
+      <c r="J22" s="43"/>
       <c r="K22" cm="1">
         <f t="array" aca="1" ref="K22" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*2*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*2*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*2*24)</f>
         <v>0</v>
@@ -1594,7 +1575,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J23" s="42"/>
+      <c r="J23" s="43"/>
       <c r="K23" cm="1">
         <f t="array" aca="1" ref="K23" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1618,7 +1599,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J24" s="42"/>
+      <c r="J24" s="43"/>
       <c r="K24" cm="1">
         <f t="array" aca="1" ref="K24" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1642,7 +1623,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J25" s="42"/>
+      <c r="J25" s="43"/>
       <c r="K25" cm="1">
         <f t="array" aca="1" ref="K25" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1666,7 +1647,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J26" s="42"/>
+      <c r="J26" s="43"/>
       <c r="K26" cm="1">
         <f t="array" aca="1" ref="K26" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1690,7 +1671,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J27" s="42"/>
+      <c r="J27" s="43"/>
       <c r="K27" cm="1">
         <f t="array" aca="1" ref="K27" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1714,7 +1695,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J28" s="42"/>
+      <c r="J28" s="43"/>
       <c r="K28" cm="1">
         <f t="array" aca="1" ref="K28" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*2*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*2*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*2*24)</f>
         <v>0</v>
@@ -1738,7 +1719,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J29" s="42"/>
+      <c r="J29" s="43"/>
       <c r="K29" cm="1">
         <f t="array" aca="1" ref="K29" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*2*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*2*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*2*24)</f>
         <v>0</v>
@@ -1762,7 +1743,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J30" s="42"/>
+      <c r="J30" s="43"/>
       <c r="K30" cm="1">
         <f t="array" aca="1" ref="K30" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*2*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*2*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*2*24)</f>
         <v>0</v>
@@ -1786,7 +1767,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J31" s="42"/>
+      <c r="J31" s="43"/>
       <c r="K31" cm="1">
         <f t="array" aca="1" ref="K31" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1810,7 +1791,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J32" s="42"/>
+      <c r="J32" s="43"/>
       <c r="K32" cm="1">
         <f t="array" aca="1" ref="K32" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1834,7 +1815,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J33" s="42"/>
+      <c r="J33" s="43"/>
       <c r="K33" cm="1">
         <f t="array" aca="1" ref="K33" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1858,7 +1839,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J34" s="42"/>
+      <c r="J34" s="43"/>
       <c r="K34" cm="1">
         <f t="array" aca="1" ref="K34" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*1.5*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*1.5*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*1.5*24)</f>
         <v>0</v>
@@ -1882,7 +1863,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J35" s="42"/>
+      <c r="J35" s="43"/>
       <c r="K35" cm="1">
         <f t="array" aca="1" ref="K35" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*2*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*2*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*2*24)</f>
         <v>0</v>
@@ -1893,7 +1874,7 @@
         <f t="shared" si="0"/>
         <v>Domingo</v>
       </c>
-      <c r="B36" s="44">
+      <c r="B36" s="40">
         <v>46173</v>
       </c>
       <c r="C36" s="27"/>
@@ -1906,7 +1887,7 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="J36" s="43"/>
+      <c r="J36" s="44"/>
       <c r="K36" cm="1">
         <f t="array" aca="1" ref="K36" ca="1">SUM((INDIRECT("D"&amp;ROW())-INDIRECT("C"&amp;ROW()))*2*24,(INDIRECT("F"&amp;ROW())-INDIRECT("E"&amp;ROW()))*2*24,(INDIRECT("H"&amp;ROW())-INDIRECT("G"&amp;ROW()))*2*24)</f>
         <v>0</v>

</xml_diff>